<commit_message>
HEID-184 changes made based on new backend
</commit_message>
<xml_diff>
--- a/public/add_product_template.xlsx
+++ b/public/add_product_template.xlsx
@@ -24,10 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="9">
-  <si>
-    <t>id</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>description</t>
   </si>
@@ -42,12 +39,6 @@
   </si>
   <si>
     <t>name</t>
-  </si>
-  <si>
-    <t>Lenovo LOQ...</t>
-  </si>
-  <si>
-    <t>Discover the Lenovo...</t>
   </si>
   <si>
     <t>image_file_name</t>
@@ -117,15 +108,13 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -406,173 +395,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5703125" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1013</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1">
-        <v>73500</v>
-      </c>
-      <c r="E2" s="1">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1">
-        <v>73500</v>
-      </c>
-      <c r="E3" s="1">
-        <v>5</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1">
-        <v>73500</v>
-      </c>
-      <c r="E4" s="1">
-        <v>5</v>
-      </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1">
-        <v>73500</v>
-      </c>
-      <c r="E5" s="1">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1">
-        <v>73500</v>
-      </c>
-      <c r="E6" s="1">
-        <v>5</v>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1">
-        <v>73500</v>
-      </c>
-      <c r="E7" s="1">
-        <v>5</v>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1">
-        <v>73500</v>
-      </c>
-      <c r="E8" s="1">
-        <v>5</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>